<commit_message>
data: publish current surveillance partitions
</commit_message>
<xml_diff>
--- a/diseases/d043/2000-2004.xlsx
+++ b/diseases/d043/2000-2004.xlsx
@@ -9286,11 +9286,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA56" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -9303,7 +9298,7 @@
       </c>
       <c r="AP56" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ56" t="inlineStr">
@@ -9313,15 +9308,15 @@
       </c>
       <c r="AS56" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU56" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV56" t="inlineStr">
@@ -9537,7 +9532,7 @@
       </c>
       <c r="AP57" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ57" t="inlineStr">
@@ -9547,15 +9542,15 @@
       </c>
       <c r="AS57" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU57" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV57" t="inlineStr">
@@ -15294,11 +15289,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA87" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -15311,7 +15301,7 @@
       </c>
       <c r="AP87" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ87" t="inlineStr">
@@ -15321,15 +15311,15 @@
       </c>
       <c r="AS87" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU87" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV87" t="inlineStr">
@@ -15545,7 +15535,7 @@
       </c>
       <c r="AP88" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ88" t="inlineStr">
@@ -15555,15 +15545,15 @@
       </c>
       <c r="AS88" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU88" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV88" t="inlineStr">
@@ -28857,11 +28847,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA157" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -28874,7 +28859,7 @@
       </c>
       <c r="AP157" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ157" t="inlineStr">
@@ -28884,15 +28869,15 @@
       </c>
       <c r="AS157" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU157" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV157" t="inlineStr">
@@ -29108,7 +29093,7 @@
       </c>
       <c r="AP158" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ158" t="inlineStr">
@@ -29118,15 +29103,15 @@
       </c>
       <c r="AS158" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU158" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV158" t="inlineStr">
@@ -36417,11 +36402,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA196" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -36434,7 +36414,7 @@
       </c>
       <c r="AP196" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ196" t="inlineStr">
@@ -36444,15 +36424,15 @@
       </c>
       <c r="AS196" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU196" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV196" t="inlineStr">
@@ -36668,7 +36648,7 @@
       </c>
       <c r="AP197" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ197" t="inlineStr">
@@ -36678,15 +36658,15 @@
       </c>
       <c r="AS197" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT197" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU197" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV197" t="inlineStr">
@@ -42420,11 +42400,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA227" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -42437,7 +42412,7 @@
       </c>
       <c r="AP227" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ227" t="inlineStr">
@@ -42447,15 +42422,15 @@
       </c>
       <c r="AS227" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU227" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV227" t="inlineStr">
@@ -42671,7 +42646,7 @@
       </c>
       <c r="AP228" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ228" t="inlineStr">
@@ -42681,15 +42656,15 @@
       </c>
       <c r="AS228" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU228" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV228" t="inlineStr">
@@ -49199,11 +49174,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA262" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -49216,7 +49186,7 @@
       </c>
       <c r="AP262" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ262" t="inlineStr">
@@ -49226,15 +49196,15 @@
       </c>
       <c r="AS262" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT262" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU262" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV262" t="inlineStr">
@@ -49450,7 +49420,7 @@
       </c>
       <c r="AP263" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ263" t="inlineStr">
@@ -49460,15 +49430,15 @@
       </c>
       <c r="AS263" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT263" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU263" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV263" t="inlineStr">
@@ -55983,11 +55953,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U297" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA297" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -56000,7 +55965,7 @@
       </c>
       <c r="AP297" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ297" t="inlineStr">
@@ -56010,15 +55975,15 @@
       </c>
       <c r="AS297" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT297" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU297" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV297" t="inlineStr">
@@ -56234,7 +56199,7 @@
       </c>
       <c r="AP298" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ298" t="inlineStr">
@@ -56244,15 +56209,15 @@
       </c>
       <c r="AS298" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT298" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU298" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV298" t="inlineStr">
@@ -62762,11 +62727,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U332" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA332" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -62779,7 +62739,7 @@
       </c>
       <c r="AP332" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ332" t="inlineStr">
@@ -62789,15 +62749,15 @@
       </c>
       <c r="AS332" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT332" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU332" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV332" t="inlineStr">
@@ -63013,7 +62973,7 @@
       </c>
       <c r="AP333" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ333" t="inlineStr">
@@ -63023,15 +62983,15 @@
       </c>
       <c r="AS333" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT333" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU333" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV333" t="inlineStr">
@@ -69934,11 +69894,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U369" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA369" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -69951,7 +69906,7 @@
       </c>
       <c r="AP369" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ369" t="inlineStr">
@@ -69961,15 +69916,15 @@
       </c>
       <c r="AS369" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT369" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU369" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV369" t="inlineStr">
@@ -70185,7 +70140,7 @@
       </c>
       <c r="AP370" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ370" t="inlineStr">
@@ -70195,15 +70150,15 @@
       </c>
       <c r="AS370" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT370" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU370" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV370" t="inlineStr">
@@ -76713,11 +76668,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U404" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA404" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -76730,7 +76680,7 @@
       </c>
       <c r="AP404" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ404" t="inlineStr">
@@ -76740,15 +76690,15 @@
       </c>
       <c r="AS404" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT404" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU404" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV404" t="inlineStr">
@@ -76964,7 +76914,7 @@
       </c>
       <c r="AP405" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ405" t="inlineStr">
@@ -76974,15 +76924,15 @@
       </c>
       <c r="AS405" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT405" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU405" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV405" t="inlineStr">
@@ -83492,11 +83442,6 @@
           <t>nbs_computed</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr">
-        <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
-        </is>
-      </c>
       <c r="AA439" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -83509,7 +83454,7 @@
       </c>
       <c r="AP439" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ439" t="inlineStr">
@@ -83519,15 +83464,15 @@
       </c>
       <c r="AS439" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT439" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU439" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV439" t="inlineStr">
@@ -83743,7 +83688,7 @@
       </c>
       <c r="AP440" t="inlineStr">
         <is>
-          <t>single_series</t>
+          <t>priority_overlay</t>
         </is>
       </c>
       <c r="AQ440" t="inlineStr">
@@ -83753,15 +83698,15 @@
       </c>
       <c r="AS440" t="inlineStr">
         <is>
-          <t>SER_CN_PROV_DC_TYPHUS</t>
+          <t>SER_CN_PROV_DC_TYPHUS; SER_CN_PROV_REPORT_TYPHUS</t>
         </is>
       </c>
       <c r="AT440" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU440" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>Retained source series are overlaid per period using their explicit source priority; lower-priority observations remain downloadable.</t>
         </is>
       </c>
       <c r="AV440" t="inlineStr">

</xml_diff>